<commit_message>
fix: repair api Excel templates
</commit_message>
<xml_diff>
--- a/docs/domestic-vat-template-apis.xlsx
+++ b/docs/domestic-vat-template-apis.xlsx
@@ -321,22 +321,20 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="27.5" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="15.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="15.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="27.5" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="13.75" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="13.75" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="13.75" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="18.75" hidden="0" customWidth="1"/>
@@ -345,104 +343,168 @@
     <x:col min="21" max="21" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="27.5" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="27.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Province</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str">
-        <x:v>TIN</x:v>
-      </x:c>
-      <x:c r="C1" s="6" t="str">
-        <x:v>Company Name</x:v>
-      </x:c>
-      <x:c r="D1" s="6" t="str">
-        <x:v>Filing Type</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
-        <x:v>Filing Period</x:v>
-      </x:c>
-      <x:c r="F1" s="6" t="str">
-        <x:v>Input Date</x:v>
-      </x:c>
-      <x:c r="G1" s="6" t="str">
-        <x:v>Description</x:v>
-      </x:c>
-      <x:c r="H1" s="6" t="str">
-        <x:v>VAT Rate %</x:v>
-      </x:c>
-      <x:c r="I1" s="3" t="str">
-        <x:v>Domestic Sale Exempt LAK</x:v>
-      </x:c>
-      <x:c r="J1" s="9" t="str">
-        <x:v>User TE</x:v>
-      </x:c>
-      <x:c r="K1" s="3" t="str">
-        <x:v>Provision Number</x:v>
-      </x:c>
-      <x:c r="L1" s="9" t="str">
-        <x:v>User Benchmark Rate</x:v>
-      </x:c>
-      <x:c r="M1" s="9" t="str">
-        <x:v>User Benchmark VAT</x:v>
-      </x:c>
-      <x:c r="N1" s="9" t="str">
-        <x:v>Use User Fallback?</x:v>
-      </x:c>
-      <x:c r="O1" s="6" t="str">
-        <x:v>System Benchmark Rate %</x:v>
-      </x:c>
-      <x:c r="P1" s="12" t="str">
-        <x:v>Sales Standard LAK</x:v>
-      </x:c>
-      <x:c r="Q1" s="12" t="str">
-        <x:v>Sales Zero Rate LAK</x:v>
-      </x:c>
-      <x:c r="R1" s="12" t="str">
-        <x:v>Total Input VAT LAK</x:v>
-      </x:c>
-      <x:c r="S1" s="12" t="str">
-        <x:v>VAT Payable LAK</x:v>
-      </x:c>
-      <x:c r="T1" s="6" t="str">
-        <x:v>VAT Credit LAK</x:v>
-      </x:c>
-      <x:c r="U1" s="6" t="str">
-        <x:v>Purchase Domestic Non-exempt LAK</x:v>
-      </x:c>
-      <x:c r="V1" s="6" t="str">
-        <x:v>Purchase Domestic Exempt LAK</x:v>
-      </x:c>
-      <x:c r="W1" s="6" t="str">
-        <x:v>Total Output VAT LAK</x:v>
-      </x:c>
-      <x:c r="X1" s="9" t="str">
-        <x:v>User Fallback Reason</x:v>
-      </x:c>
-      <x:c r="Y1" s="9" t="str">
-        <x:v>User Comment</x:v>
+      <x:c r="A1" s="3" t="inlineStr">
+        <x:is>
+          <x:t>Province</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="3" t="inlineStr">
+        <x:is>
+          <x:t>TIN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C1" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Company Name</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D1" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Filing Type</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E1" s="3" t="inlineStr">
+        <x:is>
+          <x:t>Filing Period</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F1" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Input Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G1" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Description</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H1" s="6" t="inlineStr">
+        <x:is>
+          <x:t>VAT Rate %</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I1" s="3" t="inlineStr">
+        <x:is>
+          <x:t>Domestic Sale Exempt LAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J1" s="9" t="inlineStr">
+        <x:is>
+          <x:t>User TE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K1" s="3" t="inlineStr">
+        <x:is>
+          <x:t>Provision Number</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L1" s="9" t="inlineStr">
+        <x:is>
+          <x:t>User Benchmark Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M1" s="9" t="inlineStr">
+        <x:is>
+          <x:t>User Benchmark VAT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N1" s="9" t="inlineStr">
+        <x:is>
+          <x:t>Use User Fallback?</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O1" s="6" t="inlineStr">
+        <x:is>
+          <x:t>System Benchmark Rate %</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P1" s="12" t="inlineStr">
+        <x:is>
+          <x:t>Sales Standard LAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q1" s="12" t="inlineStr">
+        <x:is>
+          <x:t>Sales Zero Rate LAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R1" s="12" t="inlineStr">
+        <x:is>
+          <x:t>Total Input VAT LAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="S1" s="12" t="inlineStr">
+        <x:is>
+          <x:t>VAT Payable LAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="T1" s="6" t="inlineStr">
+        <x:is>
+          <x:t>VAT Credit LAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="U1" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Purchase Domestic Non-exempt LAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V1" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Purchase Domestic Exempt LAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W1" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Total Output VAT LAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="X1" s="9" t="inlineStr">
+        <x:is>
+          <x:t>User Fallback Reason</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Y1" s="9" t="inlineStr">
+        <x:is>
+          <x:t>User Comment</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="20" t="str">
-        <x:v>01 | Vientiane Capital</x:v>
-      </x:c>
-      <x:c r="B2" s="20" t="str">
-        <x:v>123456789-000</x:v>
-      </x:c>
-      <x:c r="C2" s="20" t="str">
-        <x:v>Example Company Co., Ltd.</x:v>
-      </x:c>
-      <x:c r="D2" s="20" t="str">
-        <x:v>Monthly</x:v>
-      </x:c>
-      <x:c r="E2" s="20" t="str">
-        <x:v>05/2026</x:v>
+      <x:c r="A2" s="20" t="inlineStr">
+        <x:is>
+          <x:t>01 | Vientiane Capital</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="20" t="inlineStr">
+        <x:is>
+          <x:t>123456789-000</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="20" t="inlineStr">
+        <x:is>
+          <x:t>Example Company Co., Ltd.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D2" s="20" t="inlineStr">
+        <x:is>
+          <x:t>Monthly</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" s="20" t="inlineStr">
+        <x:is>
+          <x:t>05/2026</x:t>
+        </x:is>
       </x:c>
       <x:c r="F2" s="20"/>
-      <x:c r="G2" s="20" t="str">
-        <x:v>Domestic exempt sale</x:v>
+      <x:c r="G2" s="20" t="inlineStr">
+        <x:is>
+          <x:t>Domestic exempt sale</x:t>
+        </x:is>
       </x:c>
       <x:c r="H2" s="21" t="n">
         <x:v>10</x:v>
@@ -451,13 +513,17 @@
         <x:v>100000000</x:v>
       </x:c>
       <x:c r="J2" s="22"/>
-      <x:c r="K2" s="20" t="str">
-        <x:v>39</x:v>
+      <x:c r="K2" s="20" t="inlineStr">
+        <x:is>
+          <x:t>39</x:t>
+        </x:is>
       </x:c>
       <x:c r="L2" s="22"/>
       <x:c r="M2" s="22"/>
-      <x:c r="N2" s="20" t="str">
-        <x:v>No</x:v>
+      <x:c r="N2" s="20" t="inlineStr">
+        <x:is>
+          <x:t>No</x:t>
+        </x:is>
       </x:c>
       <x:c r="O2" s="21" t="n">
         <x:v>10</x:v>
@@ -470,8 +536,8 @@
       <x:c r="U2" s="22"/>
       <x:c r="V2" s="22"/>
       <x:c r="W2" s="22"/>
-      <x:c r="X2" s="20" t="str"/>
-      <x:c r="Y2" s="20" t="str"/>
+      <x:c r="X2" s="20"/>
+      <x:c r="Y2" s="20"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5"/>
@@ -27447,7 +27513,6 @@
       <x:c r="Y1001" s="11"/>
     </x:row>
   </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:dataValidations count="6">
     <x:dataValidation type="list" allowBlank="0" showErrorMessage="1" showInputMessage="1" sqref="A2:A1001">
       <x:formula1>'Validation Lists'!$A$2:$A$19</x:formula1>
@@ -27468,6 +27533,7 @@
       <x:formula1>0</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -27482,231 +27548,335 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="27" t="str">
-        <x:v>Domestic VAT Import Template - Instructions</x:v>
+      <x:c r="A1" s="27" t="inlineStr">
+        <x:is>
+          <x:t>Domestic VAT Import Template - Instructions</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="30" t="str">
-        <x:v>Information Type</x:v>
-      </x:c>
-      <x:c r="B3" s="30" t="str">
-        <x:v>Color</x:v>
-      </x:c>
-      <x:c r="C3" s="30" t="str">
-        <x:v>Meaning</x:v>
-      </x:c>
-      <x:c r="D3" s="30" t="str">
-        <x:v>Examples</x:v>
+      <x:c r="A3" s="30" t="inlineStr">
+        <x:is>
+          <x:t>Information Type</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="30" t="inlineStr">
+        <x:is>
+          <x:t>Color</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" s="30" t="inlineStr">
+        <x:is>
+          <x:t>Meaning</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D3" s="30" t="inlineStr">
+        <x:is>
+          <x:t>Examples</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="5" t="str">
-        <x:v>Primary Required</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="str">
-        <x:v>Dark blue header, light blue input cells</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="str">
-        <x:v>Required for current Domestic VAT import and reporting.</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="str">
-        <x:v>Province, TIN, Filing Period, Domestic Sale Exempt, Provision Number</x:v>
+      <x:c r="A4" s="5" t="inlineStr">
+        <x:is>
+          <x:t>Primary Required</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="5" t="inlineStr">
+        <x:is>
+          <x:t>Dark blue header, light blue input cells</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="5" t="inlineStr">
+        <x:is>
+          <x:t>Required for current Domestic VAT import and reporting.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D4" s="5" t="inlineStr">
+        <x:is>
+          <x:t>Province, TIN, Filing Period, Domestic Sale Exempt, Provision Number</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="14" t="str">
-        <x:v>Primary Conditional</x:v>
-      </x:c>
-      <x:c r="B5" s="14" t="str">
-        <x:v>Medium blue header, near-white input cells</x:v>
-      </x:c>
-      <x:c r="C5" s="14" t="str">
-        <x:v>Needed only when future system calculation uses full VAT filing values.</x:v>
-      </x:c>
-      <x:c r="D5" s="14" t="str">
-        <x:v>Sales Standard, Sales Zero Rate, Total Input VAT, VAT Payable</x:v>
+      <x:c r="A5" s="14" t="inlineStr">
+        <x:is>
+          <x:t>Primary Conditional</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="14" t="inlineStr">
+        <x:is>
+          <x:t>Medium blue header, near-white input cells</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="14" t="inlineStr">
+        <x:is>
+          <x:t>Needed only when future system calculation uses full VAT filing values.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D5" s="14" t="inlineStr">
+        <x:is>
+          <x:t>Sales Standard, Sales Zero Rate, Total Input VAT, VAT Payable</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="8" t="str">
-        <x:v>Primary Optional</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="str">
-        <x:v>Slate/gray-blue header, white input cells</x:v>
-      </x:c>
-      <x:c r="C6" s="8" t="str">
-        <x:v>Official or supporting filing information useful for audit.</x:v>
-      </x:c>
-      <x:c r="D6" s="8" t="str">
-        <x:v>Company Name, Filing Type, Input Date, VAT Rate, Description</x:v>
+      <x:c r="A6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Primary Optional</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Slate/gray-blue header, white input cells</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Official or supporting filing information useful for audit.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Company Name, Filing Type, Input Date, VAT Rate, Description</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="11" t="str">
-        <x:v>User Fallback</x:v>
-      </x:c>
-      <x:c r="B7" s="11" t="str">
-        <x:v>Orange header, light amber input cells</x:v>
-      </x:c>
-      <x:c r="C7" s="11" t="str">
-        <x:v>Optional user-provided TE or benchmark values used only when primary information is incomplete.</x:v>
-      </x:c>
-      <x:c r="D7" s="11" t="str">
-        <x:v>User TE, User Benchmark Rate, User Benchmark VAT</x:v>
+      <x:c r="A7" s="11" t="inlineStr">
+        <x:is>
+          <x:t>User Fallback</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="11" t="inlineStr">
+        <x:is>
+          <x:t>Orange header, light amber input cells</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="11" t="inlineStr">
+        <x:is>
+          <x:t>Optional user-provided TE or benchmark values used only when primary information is incomplete.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D7" s="11" t="inlineStr">
+        <x:is>
+          <x:t>User TE, User Benchmark Rate, User Benchmark VAT</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="28" t="str">
-        <x:v>Protected Reference Sheets</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="str">
-        <x:v>Dark blue headers</x:v>
-      </x:c>
-      <x:c r="C8" s="28" t="str">
-        <x:v>Instructions, Validation Lists, and Data Dictionary are read-only to avoid accidental changes.</x:v>
-      </x:c>
-      <x:c r="D8" s="28" t="str">
-        <x:v>Use VAT Import for data entry.</x:v>
+      <x:c r="A8" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Protected Reference Sheets</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Dark blue headers</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Instructions, Validation Lists, and Data Dictionary are read-only to avoid accidental changes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Use VAT Import for data entry.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="28" t="str"/>
-      <x:c r="B9" s="28" t="str"/>
-      <x:c r="C9" s="28" t="str"/>
-      <x:c r="D9" s="28" t="str"/>
+      <x:c r="A9" s="28"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="30" t="str">
-        <x:v>Rule</x:v>
-      </x:c>
-      <x:c r="B10" s="30" t="str">
-        <x:v>Description</x:v>
-      </x:c>
-      <x:c r="C10" s="30" t="str"/>
-      <x:c r="D10" s="30" t="str"/>
+      <x:c r="A10" s="30" t="inlineStr">
+        <x:is>
+          <x:t>Rule</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="30" t="inlineStr">
+        <x:is>
+          <x:t>Description</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="30"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="28" t="str">
-        <x:v>Current compatibility</x:v>
-      </x:c>
-      <x:c r="B11" s="28" t="str">
-        <x:v>Columns A:K match the current Domestic VAT importer. The newer expert file uses A:I; User TE and Provision Number remain optional compatibility fields.</x:v>
-      </x:c>
-      <x:c r="C11" s="28" t="str"/>
-      <x:c r="D11" s="28" t="str"/>
+      <x:c r="A11" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Current compatibility</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Columns A:K match the current Domestic VAT importer. The newer expert file uses A:I; User TE and Provision Number remain optional compatibility fields.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="28"/>
+      <x:c r="D11" s="28"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="28" t="str">
-        <x:v>Use primary first</x:v>
-      </x:c>
-      <x:c r="B12" s="28" t="str">
-        <x:v>Enter raw exempt domestic sale and official filing fields before using fallback values.</x:v>
-      </x:c>
-      <x:c r="C12" s="28" t="str"/>
-      <x:c r="D12" s="28" t="str"/>
+      <x:c r="A12" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Use primary first</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Enter raw exempt domestic sale and official filing fields before using fallback values.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="28" t="str">
-        <x:v>No simple Excel calculations</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="str">
-        <x:v>Do not add columns that only multiply exempt sales by VAT rate. The system should calculate those values.</x:v>
-      </x:c>
-      <x:c r="C13" s="28" t="str"/>
-      <x:c r="D13" s="28" t="str"/>
+      <x:c r="A13" s="28" t="inlineStr">
+        <x:is>
+          <x:t>No simple Excel calculations</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Do not add columns that only multiply exempt sales by VAT rate. The system should calculate those values.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="28" t="str">
-        <x:v>Fallback rule</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="str">
-        <x:v>Use User TE or User Benchmark values only when agreed user judgement is required.</x:v>
-      </x:c>
-      <x:c r="C14" s="28" t="str"/>
-      <x:c r="D14" s="28" t="str"/>
+      <x:c r="A14" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Fallback rule</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Use User TE or User Benchmark values only when agreed user judgement is required.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="28" t="str">
-        <x:v>Fallback reason</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="str">
-        <x:v>Required when Use User Fallback? is Yes.</x:v>
-      </x:c>
-      <x:c r="C15" s="28" t="str"/>
-      <x:c r="D15" s="28" t="str"/>
+      <x:c r="A15" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Fallback reason</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Required when Use User Fallback? is Yes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="28" t="str">
-        <x:v>Dropdown fields</x:v>
-      </x:c>
-      <x:c r="B16" s="28" t="str">
-        <x:v>Province, Provision Number, Use User Fallback?, and User Fallback Reason should use dropdowns.</x:v>
-      </x:c>
-      <x:c r="C16" s="28" t="str"/>
-      <x:c r="D16" s="28" t="str"/>
+      <x:c r="A16" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Dropdown fields</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Province, Provision Number, Use User Fallback?, and User Fallback Reason should use dropdowns.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="28" t="str">
-        <x:v>Future calculation fields</x:v>
-      </x:c>
-      <x:c r="B17" s="28" t="str">
-        <x:v>Columns P:W support a fuller VAT calculation path but are ignored by the current importer until import_vat.php is updated.</x:v>
-      </x:c>
-      <x:c r="C17" s="28" t="str"/>
-      <x:c r="D17" s="28" t="str"/>
+      <x:c r="A17" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Future calculation fields</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Columns P:W support a fuller VAT calculation path but are ignored by the current importer until import_vat.php is updated.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="28" t="str">
-        <x:v>Mandatory fields</x:v>
-      </x:c>
-      <x:c r="B18" s="28" t="str">
-        <x:v>Province, TIN, Filing Period, Domestic Sale Exempt, and Provision Number.</x:v>
-      </x:c>
-      <x:c r="C18" s="28" t="str"/>
-      <x:c r="D18" s="28" t="str"/>
+      <x:c r="A18" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Mandatory fields</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Province, TIN, Filing Period, Domestic Sale Exempt, and Provision Number.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="28" t="str">
-        <x:v>Template version</x:v>
-      </x:c>
-      <x:c r="B19" s="28" t="str">
-        <x:v>DOMESTIC_VAT_IMPORT v1.0</x:v>
-      </x:c>
-      <x:c r="C19" s="28" t="str"/>
-      <x:c r="D19" s="28" t="str"/>
+      <x:c r="A19" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Template version</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="28" t="inlineStr">
+        <x:is>
+          <x:t>DOMESTIC_VAT_IMPORT v1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="28" t="str">
-        <x:v>Protection password</x:v>
-      </x:c>
-      <x:c r="B20" s="28" t="str">
-        <x:v>TaxETS2026</x:v>
-      </x:c>
-      <x:c r="C20" s="28" t="str">
-        <x:v>Used only to prevent accidental edits to read-only sheets.</x:v>
-      </x:c>
-      <x:c r="D20" s="28" t="str"/>
+      <x:c r="A20" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Protection password</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="28" t="inlineStr">
+        <x:is>
+          <x:t>TaxETS2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Used only to prevent accidental edits to read-only sheets.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="28"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="28" t="str">
-        <x:v>Import code note</x:v>
-      </x:c>
-      <x:c r="B21" s="28" t="str">
-        <x:v>After agreement, import_vat.php should be updated to read by header name and apply the hybrid fallback principle explicitly.</x:v>
-      </x:c>
-      <x:c r="C21" s="28" t="str"/>
-      <x:c r="D21" s="28" t="str"/>
+      <x:c r="A21" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Import code note</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" s="28" t="inlineStr">
+        <x:is>
+          <x:t>After agreement, import_vat.php should be updated to read by header name and apply the hybrid fallback principle explicitly.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="28"/>
+      <x:c r="D21" s="28"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="28" t="str">
-        <x:v>Expert file comparison</x:v>
-      </x:c>
-      <x:c r="B22" s="28" t="str">
-        <x:v>The second expert file removed calculated TE and provision columns. APIS keeps the raw-data direction and separates user fallback fields.</x:v>
-      </x:c>
-      <x:c r="C22" s="28" t="str"/>
-      <x:c r="D22" s="28" t="str"/>
+      <x:c r="A22" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Expert file comparison</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" s="28" t="inlineStr">
+        <x:is>
+          <x:t>The second expert file removed calculated TE and provision columns. APIS keeps the raw-data direction and separates user fallback fields.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="28"/>
+      <x:c r="D22" s="28"/>
     </x:row>
   </x:sheetData>
   <x:sheetProtection password="C3BC" sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
@@ -27722,542 +27892,866 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="27.5" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="27.5" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="27.5" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="53.75" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="27.5" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="15.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="53.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="24" t="str">
-        <x:v>Province Item</x:v>
-      </x:c>
-      <x:c r="B1" s="24" t="str">
-        <x:v>Province Code</x:v>
-      </x:c>
-      <x:c r="C1" s="24" t="str">
-        <x:v>Province Name</x:v>
+      <x:c r="A1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Province Item</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Province Code</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Province Name</x:t>
+        </x:is>
       </x:c>
       <x:c r="D1" s="24"/>
-      <x:c r="E1" s="24" t="str">
-        <x:v>Provision Number</x:v>
-      </x:c>
-      <x:c r="F1" s="24" t="str">
-        <x:v>Legal Basis</x:v>
-      </x:c>
-      <x:c r="G1" s="24" t="str">
-        <x:v>Type</x:v>
-      </x:c>
-      <x:c r="H1" s="24" t="str">
-        <x:v>Yes/No</x:v>
-      </x:c>
-      <x:c r="I1" s="24" t="str">
-        <x:v>Purpose</x:v>
-      </x:c>
-      <x:c r="J1" s="24" t="str">
-        <x:v>Fallback Reason</x:v>
-      </x:c>
-      <x:c r="K1" s="24" t="str">
-        <x:v>Start Date</x:v>
-      </x:c>
-      <x:c r="L1" s="24" t="str">
-        <x:v>End Date</x:v>
-      </x:c>
-      <x:c r="M1" s="24" t="str">
-        <x:v>Rate %</x:v>
+      <x:c r="E1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Provision Number</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Legal Basis</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Type</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Yes/No</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Purpose</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Fallback Reason</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Start Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>End Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M1" s="24" t="inlineStr">
+        <x:is>
+          <x:t>Rate %</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>01 | Vientiane Capital</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>01</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>Vientiane Capital</x:v>
-      </x:c>
-      <x:c r="E2" t="str">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="F2" t="str">
-        <x:v>VAT Law Art. 12.1.1</x:v>
-      </x:c>
-      <x:c r="G2" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H2" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I2" t="str">
-        <x:v>Food security</x:v>
-      </x:c>
-      <x:c r="J2" t="str"/>
-      <x:c r="K2" t="str">
-        <x:v>2010-01-01</x:v>
-      </x:c>
-      <x:c r="L2" t="str">
-        <x:v>2021-12-31</x:v>
-      </x:c>
-      <x:c r="M2" t="str">
-        <x:v>10.00</x:v>
+      <x:c r="A2" t="inlineStr">
+        <x:is>
+          <x:t>01 | Vientiane Capital</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" t="inlineStr">
+        <x:is>
+          <x:t>01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" t="inlineStr">
+        <x:is>
+          <x:t>Vientiane Capital</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" t="inlineStr">
+        <x:is>
+          <x:t>31</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F2" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G2" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H2" t="inlineStr">
+        <x:is>
+          <x:t>No</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I2" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J2"/>
+      <x:c r="K2" t="inlineStr">
+        <x:is>
+          <x:t>2010-01-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L2" t="inlineStr">
+        <x:is>
+          <x:t>2021-12-31</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M2" t="inlineStr">
+        <x:is>
+          <x:t>10.00</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>02 | Phongsaly</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>02</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>Phongsaly</x:v>
-      </x:c>
-      <x:c r="E3" t="str">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F3" t="str">
-        <x:v>VAT Law Art. 12.1.2</x:v>
-      </x:c>
-      <x:c r="G3" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H3" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="I3" t="str">
-        <x:v>Food security</x:v>
-      </x:c>
-      <x:c r="J3" t="str">
-        <x:v>Missing VAT payable</x:v>
-      </x:c>
-      <x:c r="K3" t="str">
-        <x:v>2022-01-01</x:v>
-      </x:c>
-      <x:c r="L3" t="str">
-        <x:v>2024-03-31</x:v>
-      </x:c>
-      <x:c r="M3" t="str">
-        <x:v>7.00</x:v>
+      <x:c r="A3" t="inlineStr">
+        <x:is>
+          <x:t>02 | Phongsaly</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" t="inlineStr">
+        <x:is>
+          <x:t>02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" t="inlineStr">
+        <x:is>
+          <x:t>Phongsaly</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" t="inlineStr">
+        <x:is>
+          <x:t>32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G3" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H3" t="inlineStr">
+        <x:is>
+          <x:t>Yes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I3" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J3" t="inlineStr">
+        <x:is>
+          <x:t>Missing VAT payable</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K3" t="inlineStr">
+        <x:is>
+          <x:t>2022-01-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L3" t="inlineStr">
+        <x:is>
+          <x:t>2024-03-31</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M3" t="inlineStr">
+        <x:is>
+          <x:t>7.00</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>03 | Luangnamtha</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>03</x:v>
-      </x:c>
-      <x:c r="C4" t="str">
-        <x:v>Luangnamtha</x:v>
-      </x:c>
-      <x:c r="E4" t="str">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="F4" t="str">
-        <x:v>VAT Law Art. 12.1.3</x:v>
-      </x:c>
-      <x:c r="G4" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H4" t="str">
-        <x:v>Import of: Equipment and machinery used in agriculture</x:v>
-      </x:c>
-      <x:c r="I4" t="str">
-        <x:v>Food security</x:v>
-      </x:c>
-      <x:c r="J4" t="str">
-        <x:v>Missing total input VAT</x:v>
-      </x:c>
-      <x:c r="K4" t="str">
-        <x:v>2024-04-01</x:v>
-      </x:c>
-      <x:c r="L4" t="str">
-        <x:v>2099-12-31</x:v>
-      </x:c>
-      <x:c r="M4" t="str">
-        <x:v>10.00</x:v>
+      <x:c r="A4" t="inlineStr">
+        <x:is>
+          <x:t>03 | Luangnamtha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" t="inlineStr">
+        <x:is>
+          <x:t>03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" t="inlineStr">
+        <x:is>
+          <x:t>Luangnamtha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" t="inlineStr">
+        <x:is>
+          <x:t>33</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F4" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G4" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H4" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Equipment and machinery used in agriculture</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I4" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J4" t="inlineStr">
+        <x:is>
+          <x:t>Missing total input VAT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K4" t="inlineStr">
+        <x:is>
+          <x:t>2024-04-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L4" t="inlineStr">
+        <x:is>
+          <x:t>2099-12-31</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M4" t="inlineStr">
+        <x:is>
+          <x:t>10.00</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>04 | Oudomxay</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>04</x:v>
-      </x:c>
-      <x:c r="C5" t="str">
-        <x:v>Oudomxay</x:v>
-      </x:c>
-      <x:c r="E5" t="str">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="F5" t="str">
-        <x:v>VAT Law Art. 12.1.5; IPL Art. 12</x:v>
-      </x:c>
-      <x:c r="G5" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H5" t="str">
-        <x:v>Import of: Materials [and] equipment that could not be supplied or produced in Lao PDR and machinery that are used as fixed assets and used directly in production</x:v>
-      </x:c>
-      <x:c r="I5" t="str">
-        <x:v>Investment Promotion / Export Promotion</x:v>
-      </x:c>
-      <x:c r="J5" t="str">
-        <x:v>Missing full sales split</x:v>
+      <x:c r="A5" t="inlineStr">
+        <x:is>
+          <x:t>04 | Oudomxay</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" t="inlineStr">
+        <x:is>
+          <x:t>04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" t="inlineStr">
+        <x:is>
+          <x:t>Oudomxay</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E5" t="inlineStr">
+        <x:is>
+          <x:t>34</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F5" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.5; IPL Art. 12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H5" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Materials [and] equipment that could not be supplied or produced in Lao PDR and machinery that are used as fixed assets and used directly in production</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I5" t="inlineStr">
+        <x:is>
+          <x:t>Investment Promotion / Export Promotion</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J5" t="inlineStr">
+        <x:is>
+          <x:t>Missing full sales split</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>05 | Bokeo</x:v>
-      </x:c>
-      <x:c r="B6" t="str">
-        <x:v>05</x:v>
-      </x:c>
-      <x:c r="C6" t="str">
-        <x:v>Bokeo</x:v>
-      </x:c>
-      <x:c r="E6" t="str">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="F6" t="str">
-        <x:v>VAT Law Art. 12.1.13</x:v>
-      </x:c>
-      <x:c r="G6" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H6" t="str">
-        <x:v>Import of: Animal medicines, artificial organs for transplantation for animal bodies</x:v>
-      </x:c>
-      <x:c r="I6" t="str">
-        <x:v>Food security</x:v>
-      </x:c>
-      <x:c r="J6" t="str">
-        <x:v>Special legal treatment</x:v>
+      <x:c r="A6" t="inlineStr">
+        <x:is>
+          <x:t>05 | Bokeo</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" t="inlineStr">
+        <x:is>
+          <x:t>05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" t="inlineStr">
+        <x:is>
+          <x:t>Bokeo</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" t="inlineStr">
+        <x:is>
+          <x:t>35</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F6" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H6" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Animal medicines, artificial organs for transplantation for animal bodies</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I6" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J6" t="inlineStr">
+        <x:is>
+          <x:t>Special legal treatment</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>06 | Luangprabang</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>06</x:v>
-      </x:c>
-      <x:c r="C7" t="str">
-        <x:v>Luangprabang</x:v>
-      </x:c>
-      <x:c r="E7" t="str">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F7" t="str">
-        <x:v>VAT Law Art. 12.1.14</x:v>
-      </x:c>
-      <x:c r="G7" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H7" t="str">
-        <x:v>Import of: Traditional medicines, artificial organs for transplantation for human bodies, human blood and supporting equipment for patients, the disabled and elderly</x:v>
-      </x:c>
-      <x:c r="I7" t="str">
-        <x:v>Social - Health</x:v>
-      </x:c>
-      <x:c r="J7" t="str">
-        <x:v>Legacy assessment</x:v>
+      <x:c r="A7" t="inlineStr">
+        <x:is>
+          <x:t>06 | Luangprabang</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" t="inlineStr">
+        <x:is>
+          <x:t>06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" t="inlineStr">
+        <x:is>
+          <x:t>Luangprabang</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" t="inlineStr">
+        <x:is>
+          <x:t>36</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.14</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H7" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Traditional medicines, artificial organs for transplantation for human bodies, human blood and supporting equipment for patients, the disabled and elderly</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I7" t="inlineStr">
+        <x:is>
+          <x:t>Social - Health</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J7" t="inlineStr">
+        <x:is>
+          <x:t>Legacy assessment</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>07 | Huaphanh</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>07</x:v>
-      </x:c>
-      <x:c r="C8" t="str">
-        <x:v>Huaphanh</x:v>
-      </x:c>
-      <x:c r="E8" t="str">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="F8" t="str">
-        <x:v>VAT Law Art. 12.1.15</x:v>
-      </x:c>
-      <x:c r="G8" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H8" t="str">
-        <x:v>Import of: Medical tools [and] equipment, [laboratory] equipments or wheelchairs for public services of hospitals, health care centers</x:v>
-      </x:c>
-      <x:c r="I8" t="str">
-        <x:v>Social - Health</x:v>
-      </x:c>
-      <x:c r="J8" t="str">
-        <x:v>User judgment</x:v>
+      <x:c r="A8" t="inlineStr">
+        <x:is>
+          <x:t>07 | Huaphanh</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" t="inlineStr">
+        <x:is>
+          <x:t>07</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" t="inlineStr">
+        <x:is>
+          <x:t>Huaphanh</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" t="inlineStr">
+        <x:is>
+          <x:t>37</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F8" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H8" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Medical tools [and] equipment, [laboratory] equipments or wheelchairs for public services of hospitals, health care centers</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I8" t="inlineStr">
+        <x:is>
+          <x:t>Social - Health</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J8" t="inlineStr">
+        <x:is>
+          <x:t>User judgment</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>08 | Sayaboury</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>08</x:v>
-      </x:c>
-      <x:c r="C9" t="str">
-        <x:v>Sayaboury</x:v>
-      </x:c>
-      <x:c r="E9" t="str">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="F9" t="str">
-        <x:v>VAT Law Art. 12.1.16</x:v>
-      </x:c>
-      <x:c r="G9" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H9" t="str">
-        <x:v>Import of: Vehicles serving professional activities, contributing to public benefits such as fire trucks, ambulances, vehicles equipped with repair facilities, outside television and radio broadcast vehicles and other professional vehicles</x:v>
-      </x:c>
-      <x:c r="I9" t="str">
-        <x:v>Not available on the local market</x:v>
-      </x:c>
-      <x:c r="J9" t="str">
-        <x:v>Other</x:v>
+      <x:c r="A9" t="inlineStr">
+        <x:is>
+          <x:t>08 | Sayaboury</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" t="inlineStr">
+        <x:is>
+          <x:t>08</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" t="inlineStr">
+        <x:is>
+          <x:t>Sayaboury</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" t="inlineStr">
+        <x:is>
+          <x:t>38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F9" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H9" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Vehicles serving professional activities, contributing to public benefits such as fire trucks, ambulances, vehicles equipped with repair facilities, outside television and radio broadcast vehicles and other professional vehicles</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I9" t="inlineStr">
+        <x:is>
+          <x:t>Not available on the local market</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J9" t="inlineStr">
+        <x:is>
+          <x:t>Other</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>09 | Xiengkhouang</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>09</x:v>
-      </x:c>
-      <x:c r="C10" t="str">
-        <x:v>Xiengkhouang</x:v>
-      </x:c>
-      <x:c r="E10" t="str">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="F10" t="str">
-        <x:v>VAT Law Art. 12.2.1</x:v>
-      </x:c>
-      <x:c r="G10" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H10" t="str">
-        <x:v>Domestic supply of: Unprocessed agricultural or preliminary processed products including peeled, grinded [and] milled</x:v>
-      </x:c>
-      <x:c r="I10" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A10" t="inlineStr">
+        <x:is>
+          <x:t>09 | Xiengkhouang</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" t="inlineStr">
+        <x:is>
+          <x:t>09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" t="inlineStr">
+        <x:is>
+          <x:t>Xiengkhouang</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E10" t="inlineStr">
+        <x:is>
+          <x:t>39</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F10" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H10" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: Unprocessed agricultural or preliminary processed products including peeled, grinded [and] milled</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I10" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>10 | Vientiane Province</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C11" t="str">
-        <x:v>Vientiane Province</x:v>
-      </x:c>
-      <x:c r="E11" t="str">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="F11" t="str">
-        <x:v>VAT Law Art. 12.2.2</x:v>
-      </x:c>
-      <x:c r="G11" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H11" t="str">
-        <x:v>Domestic supply of: All kinds of live or deceased animals, whole or in parts, that are unprocessed or preliminary processed to ensure freshness or non-perishability</x:v>
-      </x:c>
-      <x:c r="I11" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A11" t="inlineStr">
+        <x:is>
+          <x:t>10 | Vientiane Province</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" t="inlineStr">
+        <x:is>
+          <x:t>10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" t="inlineStr">
+        <x:is>
+          <x:t>Vientiane Province</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E11" t="inlineStr">
+        <x:is>
+          <x:t>40</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F11" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H11" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: All kinds of live or deceased animals, whole or in parts, that are unprocessed or preliminary processed to ensure freshness or non-perishability</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I11" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>11 | Borikhamxay</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C12" t="str">
-        <x:v>Borikhamxay</x:v>
-      </x:c>
-      <x:c r="E12" t="str">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="F12" t="str">
-        <x:v>VAT Law Art. 12.2.3</x:v>
-      </x:c>
-      <x:c r="G12" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H12" t="str">
-        <x:v>Domestic supply of: afforestation, plantation of industrial, fruit and medicinal trees</x:v>
-      </x:c>
-      <x:c r="I12" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A12" t="inlineStr">
+        <x:is>
+          <x:t>11 | Borikhamxay</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" t="inlineStr">
+        <x:is>
+          <x:t>11</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" t="inlineStr">
+        <x:is>
+          <x:t>Borikhamxay</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" t="inlineStr">
+        <x:is>
+          <x:t>41</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H12" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: afforestation, plantation of industrial, fruit and medicinal trees</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I12" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>12 | Khamouane</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C13" t="str">
-        <x:v>Khamouane</x:v>
-      </x:c>
-      <x:c r="E13" t="str">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="F13" t="str">
-        <x:v>VAT Law Art. 12.2.4</x:v>
-      </x:c>
-      <x:c r="G13" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H13" t="str">
-        <x:v>Domestic supply of: all types of crop seeds, animals for breeding, animal feeds, vaccines, raw materials to produce animal feeds and vaccines</x:v>
-      </x:c>
-      <x:c r="I13" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A13" t="inlineStr">
+        <x:is>
+          <x:t>12 | Khamouane</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" t="inlineStr">
+        <x:is>
+          <x:t>12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" t="inlineStr">
+        <x:is>
+          <x:t>Khamouane</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" t="inlineStr">
+        <x:is>
+          <x:t>42</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: all types of crop seeds, animals for breeding, animal feeds, vaccines, raw materials to produce animal feeds and vaccines</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I13" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>13 | Savannakhet</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C14" t="str">
-        <x:v>Savannakhet</x:v>
-      </x:c>
-      <x:c r="E14" t="str">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F14" t="str">
-        <x:v>VAT Law Art. 12.2.5</x:v>
-      </x:c>
-      <x:c r="G14" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H14" t="str">
-        <x:v>Domestic supply of: Raw materials used in the production of fertilizers, agroprocessing products, organic fertilizers, [scientific] fertilizers and pesticides that are not dangerous to the ecosystem, human and animal health and life</x:v>
-      </x:c>
-      <x:c r="I14" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A14" t="inlineStr">
+        <x:is>
+          <x:t>13 | Savannakhet</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" t="inlineStr">
+        <x:is>
+          <x:t>13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" t="inlineStr">
+        <x:is>
+          <x:t>Savannakhet</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" t="inlineStr">
+        <x:is>
+          <x:t>43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H14" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: Raw materials used in the production of fertilizers, agroprocessing products, organic fertilizers, [scientific] fertilizers and pesticides that are not dangerous to the ecosystem, human and animal health and life</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I14" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>14 | Saravanh</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C15" t="str">
-        <x:v>Saravanh</x:v>
-      </x:c>
-      <x:c r="E15" t="str">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="F15" t="str">
-        <x:v>VAT Law Art. 12.2.7</x:v>
-      </x:c>
-      <x:c r="G15" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H15" t="str">
-        <x:v>Domestic supply of: equipment and machinery used in agricultural activities</x:v>
-      </x:c>
-      <x:c r="I15" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A15" t="inlineStr">
+        <x:is>
+          <x:t>14 | Saravanh</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" t="inlineStr">
+        <x:is>
+          <x:t>14</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" t="inlineStr">
+        <x:is>
+          <x:t>Saravanh</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" t="inlineStr">
+        <x:is>
+          <x:t>44</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H15" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: equipment and machinery used in agricultural activities</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I15" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>15 | Xekong</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
-        <x:v>Xekong</x:v>
-      </x:c>
-      <x:c r="E16" t="str">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="F16" t="str">
-        <x:v>VAT Law Art. 12.2.11</x:v>
-      </x:c>
-      <x:c r="G16" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H16" t="str">
-        <x:v>Domestic supply of: textbooks and learning materials</x:v>
-      </x:c>
-      <x:c r="I16" t="str">
-        <x:v>Social - Education</x:v>
+      <x:c r="A16" t="inlineStr">
+        <x:is>
+          <x:t>15 | Xekong</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" t="inlineStr">
+        <x:is>
+          <x:t>15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" t="inlineStr">
+        <x:is>
+          <x:t>Xekong</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E16" t="inlineStr">
+        <x:is>
+          <x:t>45</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.11</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H16" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: textbooks and learning materials</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I16" t="inlineStr">
+        <x:is>
+          <x:t>Social - Education</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>16 | Champasak</x:v>
-      </x:c>
-      <x:c r="B17" t="str">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C17" t="str">
-        <x:v>Champasak</x:v>
-      </x:c>
-      <x:c r="E17" t="str">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F17" t="str">
-        <x:v>VAT Law Art. 12.2.13</x:v>
-      </x:c>
-      <x:c r="G17" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H17" t="str">
-        <x:v>The supply of education services by e.g. childcare centres, kindergartens, primary and secondary schools, vocational schools, colleges, academies, universities, sporting and athletic schools</x:v>
-      </x:c>
-      <x:c r="I17" t="str">
-        <x:v>Social - Education</x:v>
+      <x:c r="A17" t="inlineStr">
+        <x:is>
+          <x:t>16 | Champasak</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" t="inlineStr">
+        <x:is>
+          <x:t>16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" t="inlineStr">
+        <x:is>
+          <x:t>Champasak</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E17" t="inlineStr">
+        <x:is>
+          <x:t>46</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F17" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H17" t="inlineStr">
+        <x:is>
+          <x:t>The supply of education services by e.g. childcare centres, kindergartens, primary and secondary schools, vocational schools, colleges, academies, universities, sporting and athletic schools</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I17" t="inlineStr">
+        <x:is>
+          <x:t>Social - Education</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>17 | Attapeu</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C18" t="str">
-        <x:v>Attapeu</x:v>
+      <x:c r="A18" t="inlineStr">
+        <x:is>
+          <x:t>17 | Attapeu</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" t="inlineStr">
+        <x:is>
+          <x:t>17</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" t="inlineStr">
+        <x:is>
+          <x:t>Attapeu</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>18 | Xaisomboun</x:v>
-      </x:c>
-      <x:c r="B19" t="str">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C19" t="str">
-        <x:v>Xaisomboun</x:v>
+      <x:c r="A19" t="inlineStr">
+        <x:is>
+          <x:t>18 | Xaisomboun</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" t="inlineStr">
+        <x:is>
+          <x:t>18</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" t="inlineStr">
+        <x:is>
+          <x:t>Xaisomboun</x:t>
+        </x:is>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -28271,518 +28765,826 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="27.5" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="27.5" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="27.5" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="53.75" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="32.5" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="15.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="53.75" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="32.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="26" t="str">
-        <x:v>Province Code</x:v>
-      </x:c>
-      <x:c r="B1" s="26" t="str">
-        <x:v>Province Name</x:v>
-      </x:c>
-      <x:c r="C1" s="26" t="str">
-        <x:v>Dropdown Value</x:v>
+      <x:c r="A1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>Province Code</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>Province Name</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>Dropdown Value</x:t>
+        </x:is>
       </x:c>
       <x:c r="D1" s="26"/>
-      <x:c r="E1" s="26" t="str">
-        <x:v>Provision Number</x:v>
-      </x:c>
-      <x:c r="F1" s="26" t="str">
-        <x:v>Legal Basis</x:v>
-      </x:c>
-      <x:c r="G1" s="26" t="str">
-        <x:v>Type</x:v>
-      </x:c>
-      <x:c r="H1" s="26" t="str">
-        <x:v>Description</x:v>
-      </x:c>
-      <x:c r="I1" s="26" t="str">
-        <x:v>Purpose</x:v>
+      <x:c r="E1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>Provision Number</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>Legal Basis</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>Type</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>Description</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>Purpose</x:t>
+        </x:is>
       </x:c>
       <x:c r="J1" s="26"/>
-      <x:c r="K1" s="26" t="str">
-        <x:v>Start Date</x:v>
-      </x:c>
-      <x:c r="L1" s="26" t="str">
-        <x:v>End Date</x:v>
-      </x:c>
-      <x:c r="M1" s="26" t="str">
-        <x:v>VAT Rate %</x:v>
+      <x:c r="K1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>Start Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>End Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M1" s="26" t="inlineStr">
+        <x:is>
+          <x:t>VAT Rate %</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>01</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>Vientiane Capital</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>01 | Vientiane Capital</x:v>
-      </x:c>
-      <x:c r="E2" t="str">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="F2" t="str">
-        <x:v>VAT Law Art. 12.1.1</x:v>
-      </x:c>
-      <x:c r="G2" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H2" t="str">
-        <x:v>Import of: all types of crop seeds, animals for breeding, animal sperms, vaccines, equipment and liquid nitrogen for storing vaccines and animal sperms, animal feeds, raw materials to produce animal feeds and vaccines</x:v>
-      </x:c>
-      <x:c r="I2" t="str">
-        <x:v>Food security</x:v>
-      </x:c>
-      <x:c r="K2" t="str">
-        <x:v>2010-01-01</x:v>
-      </x:c>
-      <x:c r="L2" t="str">
-        <x:v>2021-12-31</x:v>
-      </x:c>
-      <x:c r="M2" t="str">
-        <x:v>10.00</x:v>
+      <x:c r="A2" t="inlineStr">
+        <x:is>
+          <x:t>01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" t="inlineStr">
+        <x:is>
+          <x:t>Vientiane Capital</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" t="inlineStr">
+        <x:is>
+          <x:t>01 | Vientiane Capital</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" t="inlineStr">
+        <x:is>
+          <x:t>31</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F2" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G2" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H2" t="inlineStr">
+        <x:is>
+          <x:t>Import of: all types of crop seeds, animals for breeding, animal sperms, vaccines, equipment and liquid nitrogen for storing vaccines and animal sperms, animal feeds, raw materials to produce animal feeds and vaccines</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I2" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K2" t="inlineStr">
+        <x:is>
+          <x:t>2010-01-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L2" t="inlineStr">
+        <x:is>
+          <x:t>2021-12-31</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M2" t="inlineStr">
+        <x:is>
+          <x:t>10.00</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>02</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>Phongsaly</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>02 | Phongsaly</x:v>
-      </x:c>
-      <x:c r="E3" t="str">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F3" t="str">
-        <x:v>VAT Law Art. 12.1.2</x:v>
-      </x:c>
-      <x:c r="G3" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H3" t="str">
-        <x:v>Import of: Raw materials used in the production of fertilizers, agro-processing products, organic fertilizers, [scientific] fertilizers [and] pesticides that are not dangerous to the ecosystem, human and animal health and life</x:v>
-      </x:c>
-      <x:c r="I3" t="str">
-        <x:v>Food security</x:v>
-      </x:c>
-      <x:c r="K3" t="str">
-        <x:v>2022-01-01</x:v>
-      </x:c>
-      <x:c r="L3" t="str">
-        <x:v>2024-03-31</x:v>
-      </x:c>
-      <x:c r="M3" t="str">
-        <x:v>7.00</x:v>
+      <x:c r="A3" t="inlineStr">
+        <x:is>
+          <x:t>02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" t="inlineStr">
+        <x:is>
+          <x:t>Phongsaly</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" t="inlineStr">
+        <x:is>
+          <x:t>02 | Phongsaly</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" t="inlineStr">
+        <x:is>
+          <x:t>32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G3" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H3" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Raw materials used in the production of fertilizers, agro-processing products, organic fertilizers, [scientific] fertilizers [and] pesticides that are not dangerous to the ecosystem, human and animal health and life</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I3" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K3" t="inlineStr">
+        <x:is>
+          <x:t>2022-01-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L3" t="inlineStr">
+        <x:is>
+          <x:t>2024-03-31</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M3" t="inlineStr">
+        <x:is>
+          <x:t>7.00</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>03</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>Luangnamtha</x:v>
-      </x:c>
-      <x:c r="C4" t="str">
-        <x:v>03 | Luangnamtha</x:v>
-      </x:c>
-      <x:c r="E4" t="str">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="F4" t="str">
-        <x:v>VAT Law Art. 12.1.3</x:v>
-      </x:c>
-      <x:c r="G4" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H4" t="str">
-        <x:v>Import of: Equipment and machinery used in agriculture</x:v>
-      </x:c>
-      <x:c r="I4" t="str">
-        <x:v>Food security</x:v>
-      </x:c>
-      <x:c r="K4" t="str">
-        <x:v>2024-04-01</x:v>
-      </x:c>
-      <x:c r="L4" t="str">
-        <x:v>2099-12-31</x:v>
-      </x:c>
-      <x:c r="M4" t="str">
-        <x:v>10.00</x:v>
+      <x:c r="A4" t="inlineStr">
+        <x:is>
+          <x:t>03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" t="inlineStr">
+        <x:is>
+          <x:t>Luangnamtha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" t="inlineStr">
+        <x:is>
+          <x:t>03 | Luangnamtha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" t="inlineStr">
+        <x:is>
+          <x:t>33</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F4" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G4" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H4" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Equipment and machinery used in agriculture</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I4" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K4" t="inlineStr">
+        <x:is>
+          <x:t>2024-04-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L4" t="inlineStr">
+        <x:is>
+          <x:t>2099-12-31</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M4" t="inlineStr">
+        <x:is>
+          <x:t>10.00</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>04</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>Oudomxay</x:v>
-      </x:c>
-      <x:c r="C5" t="str">
-        <x:v>04 | Oudomxay</x:v>
-      </x:c>
-      <x:c r="E5" t="str">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="F5" t="str">
-        <x:v>VAT Law Art. 12.1.5; IPL Art. 12</x:v>
-      </x:c>
-      <x:c r="G5" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H5" t="str">
-        <x:v>Import of: Materials [and] equipment that could not be supplied or produced in Lao PDR and machinery that are used as fixed assets and used directly in production</x:v>
-      </x:c>
-      <x:c r="I5" t="str">
-        <x:v>Investment Promotion / Export Promotion</x:v>
+      <x:c r="A5" t="inlineStr">
+        <x:is>
+          <x:t>04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" t="inlineStr">
+        <x:is>
+          <x:t>Oudomxay</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" t="inlineStr">
+        <x:is>
+          <x:t>04 | Oudomxay</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E5" t="inlineStr">
+        <x:is>
+          <x:t>34</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F5" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.5; IPL Art. 12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H5" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Materials [and] equipment that could not be supplied or produced in Lao PDR and machinery that are used as fixed assets and used directly in production</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I5" t="inlineStr">
+        <x:is>
+          <x:t>Investment Promotion / Export Promotion</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>05</x:v>
-      </x:c>
-      <x:c r="B6" t="str">
-        <x:v>Bokeo</x:v>
-      </x:c>
-      <x:c r="C6" t="str">
-        <x:v>05 | Bokeo</x:v>
-      </x:c>
-      <x:c r="E6" t="str">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="F6" t="str">
-        <x:v>VAT Law Art. 12.1.13</x:v>
-      </x:c>
-      <x:c r="G6" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H6" t="str">
-        <x:v>Import of: Animal medicines, artificial organs for transplantation for animal bodies</x:v>
-      </x:c>
-      <x:c r="I6" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A6" t="inlineStr">
+        <x:is>
+          <x:t>05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" t="inlineStr">
+        <x:is>
+          <x:t>Bokeo</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" t="inlineStr">
+        <x:is>
+          <x:t>05 | Bokeo</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" t="inlineStr">
+        <x:is>
+          <x:t>35</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F6" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H6" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Animal medicines, artificial organs for transplantation for animal bodies</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I6" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>06</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>Luangprabang</x:v>
-      </x:c>
-      <x:c r="C7" t="str">
-        <x:v>06 | Luangprabang</x:v>
-      </x:c>
-      <x:c r="E7" t="str">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F7" t="str">
-        <x:v>VAT Law Art. 12.1.14</x:v>
-      </x:c>
-      <x:c r="G7" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H7" t="str">
-        <x:v>Import of: Traditional medicines, artificial organs for transplantation for human bodies, human blood and supporting equipment for patients, the disabled and elderly</x:v>
-      </x:c>
-      <x:c r="I7" t="str">
-        <x:v>Social - Health</x:v>
+      <x:c r="A7" t="inlineStr">
+        <x:is>
+          <x:t>06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" t="inlineStr">
+        <x:is>
+          <x:t>Luangprabang</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" t="inlineStr">
+        <x:is>
+          <x:t>06 | Luangprabang</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" t="inlineStr">
+        <x:is>
+          <x:t>36</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.14</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H7" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Traditional medicines, artificial organs for transplantation for human bodies, human blood and supporting equipment for patients, the disabled and elderly</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I7" t="inlineStr">
+        <x:is>
+          <x:t>Social - Health</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>07</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>Huaphanh</x:v>
-      </x:c>
-      <x:c r="C8" t="str">
-        <x:v>07 | Huaphanh</x:v>
-      </x:c>
-      <x:c r="E8" t="str">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="F8" t="str">
-        <x:v>VAT Law Art. 12.1.15</x:v>
-      </x:c>
-      <x:c r="G8" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H8" t="str">
-        <x:v>Import of: Medical tools [and] equipment, [laboratory] equipments or wheelchairs for public services of hospitals, health care centers</x:v>
-      </x:c>
-      <x:c r="I8" t="str">
-        <x:v>Social - Health</x:v>
+      <x:c r="A8" t="inlineStr">
+        <x:is>
+          <x:t>07</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" t="inlineStr">
+        <x:is>
+          <x:t>Huaphanh</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" t="inlineStr">
+        <x:is>
+          <x:t>07 | Huaphanh</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" t="inlineStr">
+        <x:is>
+          <x:t>37</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F8" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H8" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Medical tools [and] equipment, [laboratory] equipments or wheelchairs for public services of hospitals, health care centers</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I8" t="inlineStr">
+        <x:is>
+          <x:t>Social - Health</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>08</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>Sayaboury</x:v>
-      </x:c>
-      <x:c r="C9" t="str">
-        <x:v>08 | Sayaboury</x:v>
-      </x:c>
-      <x:c r="E9" t="str">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="F9" t="str">
-        <x:v>VAT Law Art. 12.1.16</x:v>
-      </x:c>
-      <x:c r="G9" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H9" t="str">
-        <x:v>Import of: Vehicles serving professional activities, contributing to public benefits such as fire trucks, ambulances, vehicles equipped with repair facilities, outside television and radio broadcast vehicles and other professional vehicles</x:v>
-      </x:c>
-      <x:c r="I9" t="str">
-        <x:v>Not available on the local market</x:v>
+      <x:c r="A9" t="inlineStr">
+        <x:is>
+          <x:t>08</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" t="inlineStr">
+        <x:is>
+          <x:t>Sayaboury</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" t="inlineStr">
+        <x:is>
+          <x:t>08 | Sayaboury</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" t="inlineStr">
+        <x:is>
+          <x:t>38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F9" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.1.16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H9" t="inlineStr">
+        <x:is>
+          <x:t>Import of: Vehicles serving professional activities, contributing to public benefits such as fire trucks, ambulances, vehicles equipped with repair facilities, outside television and radio broadcast vehicles and other professional vehicles</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I9" t="inlineStr">
+        <x:is>
+          <x:t>Not available on the local market</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>09</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>Xiengkhouang</x:v>
-      </x:c>
-      <x:c r="C10" t="str">
-        <x:v>09 | Xiengkhouang</x:v>
-      </x:c>
-      <x:c r="E10" t="str">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="F10" t="str">
-        <x:v>VAT Law Art. 12.2.1</x:v>
-      </x:c>
-      <x:c r="G10" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H10" t="str">
-        <x:v>Domestic supply of: Unprocessed agricultural or preliminary processed products including peeled, grinded [and] milled</x:v>
-      </x:c>
-      <x:c r="I10" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A10" t="inlineStr">
+        <x:is>
+          <x:t>09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" t="inlineStr">
+        <x:is>
+          <x:t>Xiengkhouang</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" t="inlineStr">
+        <x:is>
+          <x:t>09 | Xiengkhouang</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E10" t="inlineStr">
+        <x:is>
+          <x:t>39</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F10" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H10" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: Unprocessed agricultural or preliminary processed products including peeled, grinded [and] milled</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I10" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>Vientiane Province</x:v>
-      </x:c>
-      <x:c r="C11" t="str">
-        <x:v>10 | Vientiane Province</x:v>
-      </x:c>
-      <x:c r="E11" t="str">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="F11" t="str">
-        <x:v>VAT Law Art. 12.2.2</x:v>
-      </x:c>
-      <x:c r="G11" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H11" t="str">
-        <x:v>Domestic supply of: All kinds of live or deceased animals, whole or in parts, that are unprocessed or preliminary processed to ensure freshness or non-perishability</x:v>
-      </x:c>
-      <x:c r="I11" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A11" t="inlineStr">
+        <x:is>
+          <x:t>10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" t="inlineStr">
+        <x:is>
+          <x:t>Vientiane Province</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" t="inlineStr">
+        <x:is>
+          <x:t>10 | Vientiane Province</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E11" t="inlineStr">
+        <x:is>
+          <x:t>40</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F11" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H11" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: All kinds of live or deceased animals, whole or in parts, that are unprocessed or preliminary processed to ensure freshness or non-perishability</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I11" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:v>Borikhamxay</x:v>
-      </x:c>
-      <x:c r="C12" t="str">
-        <x:v>11 | Borikhamxay</x:v>
-      </x:c>
-      <x:c r="E12" t="str">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="F12" t="str">
-        <x:v>VAT Law Art. 12.2.3</x:v>
-      </x:c>
-      <x:c r="G12" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H12" t="str">
-        <x:v>Domestic supply of: afforestation, plantation of industrial, fruit and medicinal trees</x:v>
-      </x:c>
-      <x:c r="I12" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A12" t="inlineStr">
+        <x:is>
+          <x:t>11</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" t="inlineStr">
+        <x:is>
+          <x:t>Borikhamxay</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" t="inlineStr">
+        <x:is>
+          <x:t>11 | Borikhamxay</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" t="inlineStr">
+        <x:is>
+          <x:t>41</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H12" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: afforestation, plantation of industrial, fruit and medicinal trees</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I12" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>Khamouane</x:v>
-      </x:c>
-      <x:c r="C13" t="str">
-        <x:v>12 | Khamouane</x:v>
-      </x:c>
-      <x:c r="E13" t="str">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="F13" t="str">
-        <x:v>VAT Law Art. 12.2.4</x:v>
-      </x:c>
-      <x:c r="G13" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H13" t="str">
-        <x:v>Domestic supply of: all types of crop seeds, animals for breeding, animal feeds, vaccines, raw materials to produce animal feeds and vaccines</x:v>
-      </x:c>
-      <x:c r="I13" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A13" t="inlineStr">
+        <x:is>
+          <x:t>12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" t="inlineStr">
+        <x:is>
+          <x:t>Khamouane</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" t="inlineStr">
+        <x:is>
+          <x:t>12 | Khamouane</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" t="inlineStr">
+        <x:is>
+          <x:t>42</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: all types of crop seeds, animals for breeding, animal feeds, vaccines, raw materials to produce animal feeds and vaccines</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I13" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>Savannakhet</x:v>
-      </x:c>
-      <x:c r="C14" t="str">
-        <x:v>13 | Savannakhet</x:v>
-      </x:c>
-      <x:c r="E14" t="str">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F14" t="str">
-        <x:v>VAT Law Art. 12.2.5</x:v>
-      </x:c>
-      <x:c r="G14" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H14" t="str">
-        <x:v>Domestic supply of: Raw materials used in the production of fertilizers, agroprocessing products, organic fertilizers, [scientific] fertilizers and pesticides that are not dangerous to the ecosystem, human and animal health and life</x:v>
-      </x:c>
-      <x:c r="I14" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A14" t="inlineStr">
+        <x:is>
+          <x:t>13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" t="inlineStr">
+        <x:is>
+          <x:t>Savannakhet</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" t="inlineStr">
+        <x:is>
+          <x:t>13 | Savannakhet</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" t="inlineStr">
+        <x:is>
+          <x:t>43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H14" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: Raw materials used in the production of fertilizers, agroprocessing products, organic fertilizers, [scientific] fertilizers and pesticides that are not dangerous to the ecosystem, human and animal health and life</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I14" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>Saravanh</x:v>
-      </x:c>
-      <x:c r="C15" t="str">
-        <x:v>14 | Saravanh</x:v>
-      </x:c>
-      <x:c r="E15" t="str">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="F15" t="str">
-        <x:v>VAT Law Art. 12.2.7</x:v>
-      </x:c>
-      <x:c r="G15" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H15" t="str">
-        <x:v>Domestic supply of: equipment and machinery used in agricultural activities</x:v>
-      </x:c>
-      <x:c r="I15" t="str">
-        <x:v>Food security</x:v>
+      <x:c r="A15" t="inlineStr">
+        <x:is>
+          <x:t>14</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" t="inlineStr">
+        <x:is>
+          <x:t>Saravanh</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" t="inlineStr">
+        <x:is>
+          <x:t>14 | Saravanh</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" t="inlineStr">
+        <x:is>
+          <x:t>44</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H15" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: equipment and machinery used in agricultural activities</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I15" t="inlineStr">
+        <x:is>
+          <x:t>Food security</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>Xekong</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
-        <x:v>15 | Xekong</x:v>
-      </x:c>
-      <x:c r="E16" t="str">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="F16" t="str">
-        <x:v>VAT Law Art. 12.2.11</x:v>
-      </x:c>
-      <x:c r="G16" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H16" t="str">
-        <x:v>Domestic supply of: textbooks and learning materials</x:v>
-      </x:c>
-      <x:c r="I16" t="str">
-        <x:v>Social - Education</x:v>
+      <x:c r="A16" t="inlineStr">
+        <x:is>
+          <x:t>15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" t="inlineStr">
+        <x:is>
+          <x:t>Xekong</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" t="inlineStr">
+        <x:is>
+          <x:t>15 | Xekong</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E16" t="inlineStr">
+        <x:is>
+          <x:t>45</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.11</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H16" t="inlineStr">
+        <x:is>
+          <x:t>Domestic supply of: textbooks and learning materials</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I16" t="inlineStr">
+        <x:is>
+          <x:t>Social - Education</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B17" t="str">
-        <x:v>Champasak</x:v>
-      </x:c>
-      <x:c r="C17" t="str">
-        <x:v>16 | Champasak</x:v>
-      </x:c>
-      <x:c r="E17" t="str">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F17" t="str">
-        <x:v>VAT Law Art. 12.2.13</x:v>
-      </x:c>
-      <x:c r="G17" t="str">
-        <x:v>Exemption</x:v>
-      </x:c>
-      <x:c r="H17" t="str">
-        <x:v>The supply of education services by e.g. childcare centres, kindergartens, primary and secondary schools, vocational schools, colleges, academies, universities, sporting and athletic schools</x:v>
-      </x:c>
-      <x:c r="I17" t="str">
-        <x:v>Social - Education</x:v>
+      <x:c r="A17" t="inlineStr">
+        <x:is>
+          <x:t>16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" t="inlineStr">
+        <x:is>
+          <x:t>Champasak</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" t="inlineStr">
+        <x:is>
+          <x:t>16 | Champasak</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E17" t="inlineStr">
+        <x:is>
+          <x:t>46</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F17" t="inlineStr">
+        <x:is>
+          <x:t>VAT Law Art. 12.2.13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" t="inlineStr">
+        <x:is>
+          <x:t>Exemption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H17" t="inlineStr">
+        <x:is>
+          <x:t>The supply of education services by e.g. childcare centres, kindergartens, primary and secondary schools, vocational schools, colleges, academies, universities, sporting and athletic schools</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I17" t="inlineStr">
+        <x:is>
+          <x:t>Social - Education</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>Attapeu</x:v>
-      </x:c>
-      <x:c r="C18" t="str">
-        <x:v>17 | Attapeu</x:v>
+      <x:c r="A18" t="inlineStr">
+        <x:is>
+          <x:t>17</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" t="inlineStr">
+        <x:is>
+          <x:t>Attapeu</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" t="inlineStr">
+        <x:is>
+          <x:t>17 | Attapeu</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B19" t="str">
-        <x:v>Xaisomboun</x:v>
-      </x:c>
-      <x:c r="C19" t="str">
-        <x:v>18 | Xaisomboun</x:v>
+      <x:c r="A19" t="inlineStr">
+        <x:is>
+          <x:t>18</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" t="inlineStr">
+        <x:is>
+          <x:t>Xaisomboun</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" t="inlineStr">
+        <x:is>
+          <x:t>18 | Xaisomboun</x:t>
+        </x:is>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -28802,31 +29604,47 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="31" t="str">
-        <x:v>Version</x:v>
-      </x:c>
-      <x:c r="B1" s="31" t="str">
-        <x:v>Date</x:v>
-      </x:c>
-      <x:c r="C1" s="31" t="str">
-        <x:v>Owner</x:v>
-      </x:c>
-      <x:c r="D1" s="31" t="str">
-        <x:v>Change</x:v>
+      <x:c r="A1" s="31" t="inlineStr">
+        <x:is>
+          <x:t>Version</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="31" t="inlineStr">
+        <x:is>
+          <x:t>Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C1" s="31" t="inlineStr">
+        <x:is>
+          <x:t>Owner</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D1" s="31" t="inlineStr">
+        <x:is>
+          <x:t>Change</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="28" t="str">
-        <x:v>1.0</x:v>
-      </x:c>
-      <x:c r="B2" s="28" t="str">
-        <x:v>2026-06-05</x:v>
-      </x:c>
-      <x:c r="C2" s="28" t="str">
-        <x:v>APIS / Tax-ETS</x:v>
-      </x:c>
-      <x:c r="D2" s="28" t="str">
-        <x:v>Initial recommended Domestic VAT template with current-compatible A:K and structured fallback/future calculation fields.</x:v>
+      <x:c r="A2" s="28" t="inlineStr">
+        <x:is>
+          <x:t>1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="28" t="inlineStr">
+        <x:is>
+          <x:t>2026-06-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="28" t="inlineStr">
+        <x:is>
+          <x:t>APIS / Tax-ETS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D2" s="28" t="inlineStr">
+        <x:is>
+          <x:t>Initial recommended Domestic VAT template with current-compatible A:K and structured fallback/future calculation fields.</x:t>
+        </x:is>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>